<commit_message>
Refresh Shiny app data 2026-08-04 13:22
</commit_message>
<xml_diff>
--- a/____EvoM1_TraitTable/cellcounts_selected.xlsx
+++ b/____EvoM1_TraitTable/cellcounts_selected.xlsx
@@ -21409,13 +21409,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAB85173-34EB-484A-86D1-B9560DAB64ED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{452BDA5A-15E6-4D20-990A-922D630F3BE4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28828D40-3F80-4F12-80D1-3CF2675CE1FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8DB2144-3008-4070-9F88-332101920C12}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5FBFD39-B8D9-4C52-8F6E-6097113112F9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{427CC5EF-4D12-46A0-9150-6EDA708C1A47}"/>
 </file>
</xml_diff>